<commit_message>
Minor updates to HCX control defaults.
</commit_message>
<xml_diff>
--- a/security-configuration-hardening-guide/hcx/4.11/vmware-hcx-security-configuration-guide-411-controls.xlsx
+++ b/security-configuration-hardening-guide/hcx/4.11/vmware-hcx-security-configuration-guide-411-controls.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vmware\Projects\Security Configuration Guide\Security Configuration Guide 9\WORKING COPY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vcf-security-and-compliance-guidelines\security-configuration-hardening-guide\hcx\4.11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8534FF6C-1A22-4EB2-AEC6-B958755491DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E33B40-B4B6-4820-8380-652862006FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1485" yWindow="525" windowWidth="49725" windowHeight="21120" xr2:uid="{378E67A8-D089-4FA6-9DFE-D37B9D846B86}"/>
+    <workbookView xWindow="2004" yWindow="1548" windowWidth="56784" windowHeight="23520" xr2:uid="{378E67A8-D089-4FA6-9DFE-D37B9D846B86}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="145">
   <si>
     <t>See the included documentation for important guidance and instructions.</t>
   </si>
@@ -569,153 +569,7 @@
     <t>Disabled</t>
   </si>
   <si>
-    <t>REST API Assessment</t>
-  </si>
-  <si>
-    <t>REST API Remediation</t>
-  </si>
-  <si>
     <t xml:space="preserve">All HCX appliances (Cloud, Connector, NE, and IX appliances) should be configured to forward their logs to a central, remote syslog server (e.g., VCF Operations for Logs or another SIEM solution). This ensures logs are preserved and aggregated for analysis. This is configured in the VAMI of the HCX Manager/Connector. Since HCX automatically deploys other component VMs from the HCX Manager, this setting must be configured on the HCX Manager prior to deployment. If these settings are modified after the service mesh is created a "force sync" is required. Force Sync can also be performed via APIs. </t>
-  </si>
-  <si>
-    <t>1. Configure syslog server API: 
-PUT https://&lt;hcx-manager-ip&gt;:9443/system/syslogserver
-Request:
-{
-"syslogServer": "string",
-"port": "int",
-"protocol": "string",
-"secondarySyslogServer": "string",
-"secondaryPort": "int",
-"secondaryProtocol": "string"
-}
-Response:
-Success:
-{
-  "syslogServer": "string",
-  "port": "string",
-  "protocol": "string",
-  "secondarySyslogServer": "string",
-  "secondaryPort": "string",
-  "secondaryProtocol": "string"
-}
-Failure:
-{
-  "errorCode": "integer",
-  "errorMessage": "string"
-} 
-2. Force sync DP appliance API:
-POST https://&lt;hcx-manager-ip&gt;/hybridity/api/interconnect/appliances/&lt;appliance-id&gt;/forceSync?local=&lt;boolean&gt;&amp;force=&lt;boolean&gt;
-Response:
-{
-  "data": {
-    "interconnectTaskId": "string",
-    "applianceId": "string"
-  },
-  "warnings": [
-    {
-      "code": "string",
-      "message": "string"
-    }
-  ],
-  "errors": [
-    {
-      "code": "string",
-      "message": "string"
-    }
-  ]
-}</t>
-  </si>
-  <si>
-    <t>1. Enable HA API:
-POST https://&lt;hcx-manager-ip&gt;/hybridity/api/interconnect/appliances/ha/groups
-Request:
-{
-  "appliances": ["string"],
-  "policyInfo": {
-    "policy": "string"
-  },
-  "groupId": "string"
-}
-Response:
-{
-  "data": {
-    "interconnectTaskId": "string",
-    "groupId": "string"
-  },
-  "warnings": [
-    {
-      "code": "string",
-      "message": "string"
-    }
-  ],
-  "errors": [
-    {
-      "code": "string",
-      "message": "string"
-    }
-  ]
-}
-2. Check HA status API:
-GET https://&lt;hcx-manager-ip&gt;/hybridity/api/interconnect/appliances/ha/groups/{groupId}
-Response:
-{
-  "groupId": "string",
-  "name": "string",
-  "serviceMeshId": "string",
-  "groupType": "string",
-  "groupMembers": [
-    {
-      "applianceId": "string",
-      "applianceName": "string",
-      "peerApplianceId": "string",
-      "peerApplianceName": "string",
-      "role": "string",
-      "clusterId": "string",
-      "peerClusterId": "string",
-      "location": "string"
-    }
-  ],
-  "policyInfo": {
-    "policy": "string"
-  },
-  "status": {
-    "groupState": "string",
-    "statusMessage": "string",
-    "availabilityState": "string",
-    "availabilityDescription": "string"
-  }
-}</t>
-  </si>
-  <si>
-    <t>https://{hcx-manager}:9443/components/ssh/status</t>
-  </si>
-  <si>
-    <t>POST: https://{hcx-manager}:9443/components/ssh?action=start</t>
-  </si>
-  <si>
-    <t>https://{hcx-manager}/hybridity/api/endpointInfo</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>https://{hcx-manager}:9443/system/timesettings</t>
-  </si>
-  <si>
-    <t>PUT: https://{hcx-manager}:9443/system/timesettings
-Request:
-{
-  "ntpServer": [
-    "192.19.189.10",
-    "192.19.189.10"
-  ],
-  "datetime": "12/02/2025 06:46:17",
-  "timezone": "UTC"
-}</t>
-  </si>
-  <si>
-    <t>GET: https://{hcx-manager}/hybridity/api/endpointInfo</t>
   </si>
   <si>
     <t>Control Type</t>
@@ -737,7 +591,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -846,12 +700,6 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -901,7 +749,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -939,9 +787,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -954,7 +799,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -962,119 +806,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="23">
     <dxf>
       <font>
         <b val="0"/>
@@ -1754,10 +1486,55 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -1779,31 +1556,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3695A651-C5D3-475E-B0F1-62D95BE20D6E}" name="Table1" displayName="Table1" ref="A1:V16" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowBorderDxfId="24">
-  <autoFilter ref="A1:V16" xr:uid="{3695A651-C5D3-475E-B0F1-62D95BE20D6E}"/>
-  <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{79C2AF0A-5390-4E9C-B0D5-8710D43BFCA8}" name="SCG ID" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{3A2F9A8A-E9C4-43A8-8594-3E2B9A6D5730}" name="Secure Controls_x000a_Framework ID" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{04C83ECD-7936-4E48-94C3-11B7501981A9}" name="DISA STIG ID" dataDxfId="21"/>
-    <tableColumn id="19" xr3:uid="{0C22C20C-5D4F-427F-9F5F-9E803CF25C95}" name="PCI DSS 4.0.1 ID" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{A908CAC9-5614-48A4-97C3-70CA9AC8DAFE}" name="Component_x000a_Name" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{E16C3EB7-CA62-41B0-81A3-43D994DC67B8}" name="Component Version" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{895DEAD4-BA35-4DEB-8BDB-962B3C89AD91}" name="Feature/Function" dataDxfId="17"/>
-    <tableColumn id="22" xr3:uid="{D5C7BF26-1D11-4267-B152-F653B2A06DA0}" name="Control Type" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{71DF3195-B3BB-4383-997D-CEDC42E35F5E}" name="Description/Title" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{426E1751-524C-44E0-BDFE-1D437FA86969}" name="Discussion" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{FE8DA64B-D7B6-4390-92F8-5979922A1CF8}" name="Potential Functional Impact if Default Value is Changed" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{B910FBF8-6292-4A9B-B845-87CB8C60FA3E}" name="Implementation_x000a_Priority" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{9BFF0C05-282D-4957-8499-73407BD57496}" name="Configuration Parameter" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{7AAC1EEF-6538-49BC-B64E-854CF38BD12C}" name="Installation Default Value" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{CD721173-154F-4E21-BC3D-DB2AC5F8A19C}" name="Baseline Suggested Value" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{AA97B976-1568-486E-88B7-7A4EA28C60EB}" name="Is the Default?" dataDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{02A4FA27-33A4-43FE-84CE-5CD5C84AAA7A}" name="Action Needed" dataDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{10B1F9B6-A49A-438E-AC43-8517B9CD2D77}" name="Setting Location" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{936E61C0-BF2D-4333-81AE-CF1CFBD1551E}" name="PowerCLI Command Assessment" dataDxfId="5"/>
-    <tableColumn id="21" xr3:uid="{63B187A1-3960-461E-B0B9-65EAC6B513D2}" name="PowerCLI Command Remediation" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{99812249-2B93-4E22-B188-372FD60D0537}" name="REST API Assessment" dataDxfId="3"/>
-    <tableColumn id="18" xr3:uid="{5409B494-3A6E-419E-93EC-5CDA59C980DB}" name="REST API Remediation" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3695A651-C5D3-475E-B0F1-62D95BE20D6E}" name="Table1" displayName="Table1" ref="A1:T16" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21">
+  <autoFilter ref="A1:T16" xr:uid="{3695A651-C5D3-475E-B0F1-62D95BE20D6E}"/>
+  <tableColumns count="20">
+    <tableColumn id="1" xr3:uid="{79C2AF0A-5390-4E9C-B0D5-8710D43BFCA8}" name="SCG ID" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{3A2F9A8A-E9C4-43A8-8594-3E2B9A6D5730}" name="Secure Controls_x000a_Framework ID" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{04C83ECD-7936-4E48-94C3-11B7501981A9}" name="DISA STIG ID" dataDxfId="17"/>
+    <tableColumn id="19" xr3:uid="{0C22C20C-5D4F-427F-9F5F-9E803CF25C95}" name="PCI DSS 4.0.1 ID" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{A908CAC9-5614-48A4-97C3-70CA9AC8DAFE}" name="Component_x000a_Name" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{E16C3EB7-CA62-41B0-81A3-43D994DC67B8}" name="Component Version" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{895DEAD4-BA35-4DEB-8BDB-962B3C89AD91}" name="Feature/Function" dataDxfId="13"/>
+    <tableColumn id="22" xr3:uid="{D5C7BF26-1D11-4267-B152-F653B2A06DA0}" name="Control Type" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{71DF3195-B3BB-4383-997D-CEDC42E35F5E}" name="Description/Title" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{426E1751-524C-44E0-BDFE-1D437FA86969}" name="Discussion" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{FE8DA64B-D7B6-4390-92F8-5979922A1CF8}" name="Potential Functional Impact if Default Value is Changed" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{B910FBF8-6292-4A9B-B845-87CB8C60FA3E}" name="Implementation_x000a_Priority" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{9BFF0C05-282D-4957-8499-73407BD57496}" name="Configuration Parameter" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{7AAC1EEF-6538-49BC-B64E-854CF38BD12C}" name="Installation Default Value" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{CD721173-154F-4E21-BC3D-DB2AC5F8A19C}" name="Baseline Suggested Value" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{AA97B976-1568-486E-88B7-7A4EA28C60EB}" name="Is the Default?" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{02A4FA27-33A4-43FE-84CE-5CD5C84AAA7A}" name="Action Needed" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{10B1F9B6-A49A-438E-AC43-8517B9CD2D77}" name="Setting Location" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{936E61C0-BF2D-4333-81AE-CF1CFBD1551E}" name="PowerCLI Command Assessment" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{63B187A1-3960-461E-B0B9-65EAC6B513D2}" name="PowerCLI Command Remediation" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2127,55 +1902,54 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D633219-EF3A-40A9-A077-828D0951CCAB}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="161.140625" style="18" customWidth="1"/>
-    <col min="2" max="16384" width="8.85546875" style="18"/>
+    <col min="1" max="1" width="161.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
-        <v>155</v>
+    <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
     </row>
-    <row r="7" spans="1:1" ht="105" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="105" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
     </row>
-    <row r="9" spans="1:1" ht="294" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="294" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" ht="18" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
     </row>
   </sheetData>
@@ -2185,32 +1959,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBBA3DAB-E918-4651-919A-86FFFAAB5500}">
-  <dimension ref="A1:V16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T16"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.28515625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" style="5" customWidth="1"/>
-    <col min="3" max="4" width="26.42578125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.33203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" style="5" customWidth="1"/>
+    <col min="3" max="4" width="26.44140625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="20.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19" style="5" customWidth="1"/>
-    <col min="9" max="9" width="93.140625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="104.85546875" style="5" customWidth="1"/>
-    <col min="11" max="11" width="70.7109375" style="5" customWidth="1"/>
-    <col min="12" max="12" width="23.42578125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="82.140625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="30.42578125" style="5" customWidth="1"/>
-    <col min="15" max="15" width="47.42578125" style="5" customWidth="1"/>
-    <col min="16" max="16" width="16.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="39.140625" style="5" customWidth="1"/>
-    <col min="19" max="21" width="144.7109375" style="5" customWidth="1"/>
-    <col min="22" max="22" width="143.140625" style="5" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="5"/>
+    <col min="9" max="9" width="93.109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="104.88671875" style="5" customWidth="1"/>
+    <col min="11" max="11" width="70.6640625" style="5" customWidth="1"/>
+    <col min="12" max="12" width="23.44140625" style="5" customWidth="1"/>
+    <col min="13" max="13" width="82.109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="30.44140625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="47.44140625" style="5" customWidth="1"/>
+    <col min="16" max="16" width="16.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="39.109375" style="5" customWidth="1"/>
+    <col min="19" max="20" width="144.6640625" style="5" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>4</v>
       </c>
@@ -2233,7 +2006,7 @@
         <v>9</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>10</v>
@@ -2271,14 +2044,8 @@
       <c r="T1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="U1" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="V1" s="12" t="s">
-        <v>140</v>
-      </c>
     </row>
-    <row r="2" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>50</v>
       </c>
@@ -2298,16 +2065,16 @@
         <v>57</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I2" s="9" t="s">
         <v>84</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>22</v>
@@ -2339,14 +2106,8 @@
       <c r="T2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U2" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="V2" s="13" t="s">
-        <v>142</v>
-      </c>
     </row>
-    <row r="3" spans="1:22" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>51</v>
       </c>
@@ -2366,10 +2127,10 @@
         <v>57</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I3" s="9" t="s">
         <v>85</v>
@@ -2407,14 +2168,8 @@
       <c r="T3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U3" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="V3" s="9" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="4" spans="1:22" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>99</v>
       </c>
@@ -2437,7 +2192,7 @@
         <v>102</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I4" s="10" t="s">
         <v>100</v>
@@ -2475,14 +2230,8 @@
       <c r="T4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U4" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="V4" s="9" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="5" spans="1:22" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>73</v>
       </c>
@@ -2505,7 +2254,7 @@
         <v>103</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>86</v>
@@ -2528,7 +2277,7 @@
       <c r="O5" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="P5" s="14" t="s">
+      <c r="P5" s="13" t="s">
         <v>28</v>
       </c>
       <c r="Q5" s="8" t="s">
@@ -2543,14 +2292,8 @@
       <c r="T5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U5" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="V5" s="9" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="6" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>98</v>
       </c>
@@ -2573,7 +2316,7 @@
         <v>103</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="I6" s="9" t="s">
         <v>90</v>
@@ -2611,14 +2354,8 @@
       <c r="T6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U6" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="V6" s="13" t="s">
-        <v>143</v>
-      </c>
     </row>
-    <row r="7" spans="1:22" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>52</v>
       </c>
@@ -2638,10 +2375,10 @@
         <v>57</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>91</v>
@@ -2658,16 +2395,16 @@
       <c r="M7" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="N7" s="16" t="s">
+      <c r="N7" s="15" t="s">
         <v>138</v>
       </c>
       <c r="O7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="P7" s="17" t="s">
+      <c r="P7" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="Q7" s="16" t="s">
+      <c r="Q7" s="15" t="s">
         <v>29</v>
       </c>
       <c r="R7" s="9" t="s">
@@ -2679,14 +2416,8 @@
       <c r="T7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U7" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="V7" s="13" t="s">
-        <v>145</v>
-      </c>
     </row>
-    <row r="8" spans="1:22" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>53</v>
       </c>
@@ -2706,10 +2437,10 @@
         <v>57</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>92</v>
@@ -2747,14 +2478,8 @@
       <c r="T8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U8" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="V8" s="13" t="s">
-        <v>147</v>
-      </c>
     </row>
-    <row r="9" spans="1:22" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>54</v>
       </c>
@@ -2774,10 +2499,10 @@
         <v>57</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I9" s="9" t="s">
         <v>93</v>
@@ -2815,14 +2540,8 @@
       <c r="T9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U9" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="V9" s="13" t="s">
-        <v>149</v>
-      </c>
     </row>
-    <row r="10" spans="1:22" ht="63" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>109</v>
       </c>
@@ -2842,10 +2561,10 @@
         <v>57</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>81</v>
@@ -2883,14 +2602,8 @@
       <c r="T10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U10" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="V10" s="9" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="11" spans="1:22" ht="63" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>110</v>
       </c>
@@ -2910,10 +2623,10 @@
         <v>57</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>82</v>
@@ -2951,14 +2664,8 @@
       <c r="T11" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U11" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="V11" s="9" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="12" spans="1:22" ht="63" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>111</v>
       </c>
@@ -2978,10 +2685,10 @@
         <v>57</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I12" s="9" t="s">
         <v>83</v>
@@ -3019,14 +2726,8 @@
       <c r="T12" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="U12" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="V12" s="8" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="13" spans="1:22" ht="141.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" ht="140.4" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>106</v>
       </c>
@@ -3046,10 +2747,10 @@
         <v>57</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>87</v>
@@ -3087,14 +2788,8 @@
       <c r="T13" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="U13" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="V13" s="8" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="14" spans="1:22" ht="63" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>107</v>
       </c>
@@ -3114,10 +2809,10 @@
         <v>57</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>88</v>
@@ -3155,14 +2850,8 @@
       <c r="T14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="U14" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="V14" s="8" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="15" spans="1:22" ht="63" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>108</v>
       </c>
@@ -3182,10 +2871,10 @@
         <v>57</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="I15" s="9" t="s">
         <v>89</v>
@@ -3223,14 +2912,8 @@
       <c r="T15" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="U15" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="V15" s="8" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="16" spans="1:22" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>55</v>
       </c>
@@ -3250,10 +2933,10 @@
         <v>57</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="I16" s="9" t="s">
         <v>94</v>
@@ -3279,7 +2962,7 @@
       <c r="P16" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Q16" s="15" t="s">
+      <c r="Q16" s="14" t="s">
         <v>29</v>
       </c>
       <c r="R16" s="9" t="s">
@@ -3291,15 +2974,9 @@
       <c r="T16" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="U16" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="V16" s="13" t="s">
-        <v>147</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:V16">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:T16">
     <sortCondition ref="A1:A16"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>